<commit_message>
Work Plan (3rd Month)
</commit_message>
<xml_diff>
--- a/3rd month plan.xlsx
+++ b/3rd month plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Daily-GitHub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DD73A31-6D10-4E6C-A870-C071A4B2D660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C125F8BD-B88E-45BD-9980-719CB7B062D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3379ED91-32D2-4FB5-AF2D-23BBD346235D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="36">
   <si>
     <t>Day</t>
   </si>
@@ -42,113 +42,133 @@
     <t>Platform / Task Type</t>
   </si>
   <si>
-    <t>Example Task / Problem</t>
-  </si>
-  <si>
     <t>LeetCode</t>
   </si>
   <si>
-    <t>Two Sum II – Input Array Is Sorted (#167, Easy)</t>
-  </si>
-  <si>
     <t>HackerRank</t>
   </si>
   <si>
-    <t>Solve Me First</t>
-  </si>
-  <si>
-    <t>CodeStudio</t>
-  </si>
-  <si>
-    <t>Check if String is Palindrome</t>
-  </si>
-  <si>
     <t>GeeksforGeeks</t>
   </si>
   <si>
-    <t>Find the Missing Number in Array</t>
-  </si>
-  <si>
     <t>CodeChef</t>
   </si>
   <si>
-    <t>Chef and Remissness</t>
-  </si>
-  <si>
     <t>Pandas / NumPy / SQL</t>
   </si>
   <si>
-    <t>Use Pandas to group sales data by region and compute total sales</t>
-  </si>
-  <si>
     <t>Free / Revision Day</t>
   </si>
   <si>
-    <t>Intersection of Two Linked Lists (#160, Easy)</t>
-  </si>
-  <si>
-    <t>Simple Array Sum</t>
-  </si>
-  <si>
-    <t>Find Second Largest Element</t>
-  </si>
-  <si>
-    <t>Move All Negative Elements to One Side</t>
-  </si>
-  <si>
-    <t>Chef and Stock Prices</t>
-  </si>
-  <si>
-    <t>NumPy: Create 2D array and compute row-wise sum &amp; mean</t>
-  </si>
-  <si>
-    <t>Best Time to Buy and Sell Stock (#121, Easy)</t>
-  </si>
-  <si>
-    <t>Birthday Cake Candles</t>
-  </si>
-  <si>
-    <t>Remove Duplicates from Sorted Array</t>
-  </si>
-  <si>
-    <t>Reverse Words in a String</t>
-  </si>
-  <si>
-    <t>The Lead Game</t>
-  </si>
-  <si>
-    <t>SQL: Select top 3 highest salaries from Employees table</t>
-  </si>
-  <si>
-    <t>Single Number (#136, Easy)</t>
-  </si>
-  <si>
-    <t>Compare the Triplets</t>
-  </si>
-  <si>
-    <t>Check if Array is Sorted</t>
-  </si>
-  <si>
-    <t>Missing Characters to Make a String Pangram</t>
-  </si>
-  <si>
-    <t>ATM Problem</t>
-  </si>
-  <si>
-    <t>Pandas: Merge two DataFrames and filter specific values</t>
-  </si>
-  <si>
-    <t>Climbing Stairs (#70, Easy)</t>
-  </si>
-  <si>
-    <t>Plus Minus</t>
+    <t>Task / Problem</t>
+  </si>
+  <si>
+    <t>Remove Duplicates from Sorted List (#83, Easy)</t>
+  </si>
+  <si>
+    <t>Designer PDF Viewer</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Equilibrium Point in Array</t>
+  </si>
+  <si>
+    <t>Chef and Subarrays</t>
+  </si>
+  <si>
+    <t>Pandas: Calculate correlation matrix for numeric columns</t>
+  </si>
+  <si>
+    <t>Minimum Depth of Binary Tree (#111, Easy)</t>
+  </si>
+  <si>
+    <t>Counting Sort 1</t>
+  </si>
+  <si>
+    <t>Leaders in an Array</t>
+  </si>
+  <si>
+    <t>Chef and Bored Games</t>
+  </si>
+  <si>
+    <t>Binary Search (#704, Easy)</t>
+  </si>
+  <si>
+    <t>Electronics Shop</t>
+  </si>
+  <si>
+    <t>NumPy: Generate random 3×3 matrix and normalize rows</t>
+  </si>
+  <si>
+    <t>Kadane’s Algorithm (Max Subarray Sum)</t>
+  </si>
+  <si>
+    <t>Chef and the Wildcard Matching</t>
+  </si>
+  <si>
+    <t>Move Zeroes (#283, Easy)</t>
+  </si>
+  <si>
+    <t>The Time in Words</t>
+  </si>
+  <si>
+    <t>Count the Zeros in a Sorted Binary Array</t>
+  </si>
+  <si>
+    <t>Chef and Chocolates</t>
+  </si>
+  <si>
+    <t>SQL: Write query to find 2nd highest salary using subquery</t>
+  </si>
+  <si>
+    <t>Convert Sorted Array to BST (#108, Easy)</t>
+  </si>
+  <si>
+    <t>Migratory Birds</t>
+  </si>
+  <si>
+    <t>Rearrange Array Alternately</t>
+  </si>
+  <si>
+    <t>Chef and Divisors</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pandas: Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>groupby()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> on sales by region and year</t>
+    </r>
+  </si>
+  <si>
+    <t>Pascal’s Triangle (#118, Easy)</t>
+  </si>
+  <si>
+    <t>Picking Numbers</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,6 +183,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -511,13 +536,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{357E3FA4-6155-45A2-9A7B-834BF97A7A52}">
   <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="22.33203125" customWidth="1"/>
     <col min="3" max="3" width="46.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="25.8" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -525,32 +550,32 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="25.2" customHeight="1">
       <c r="A2" s="2">
         <v>61</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="19.2" customHeight="1">
       <c r="A3" s="2">
         <v>62</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="20.399999999999999" customHeight="1">
       <c r="A4" s="2">
         <v>63</v>
       </c>
@@ -558,52 +583,54 @@
         <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="21.6" customHeight="1">
       <c r="A5" s="2">
         <v>64</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="20.399999999999999" customHeight="1">
       <c r="A6" s="2">
         <v>65</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="37.799999999999997" customHeight="1">
       <c r="A7" s="2">
         <v>66</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="22.2" customHeight="1">
       <c r="A8" s="2">
         <v>67</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:3" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:3" ht="19.2" customHeight="1">
       <c r="A9" s="2">
         <v>68</v>
       </c>
@@ -614,18 +641,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="22.2" customHeight="1">
       <c r="A10" s="2">
         <v>69</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="20.399999999999999" customHeight="1">
       <c r="A11" s="2">
         <v>70</v>
       </c>
@@ -633,63 +660,65 @@
         <v>7</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="25.2" customHeight="1">
       <c r="A12" s="2">
         <v>71</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="24" customHeight="1">
       <c r="A13" s="2">
         <v>72</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="32.4" customHeight="1">
       <c r="A14" s="2">
         <v>73</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="19.8" customHeight="1">
       <c r="A15" s="2">
         <v>74</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" spans="1:3" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="25.2" customHeight="1">
       <c r="A16" s="2">
         <v>75</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="25.2" customHeight="1">
       <c r="A17" s="2">
         <v>76</v>
       </c>
@@ -700,7 +729,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="23.4" customHeight="1">
       <c r="A18" s="2">
         <v>77</v>
       </c>
@@ -708,74 +737,76 @@
         <v>7</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="21.6" customHeight="1">
       <c r="A19" s="2">
         <v>78</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="23.4" customHeight="1">
       <c r="A20" s="2">
         <v>79</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="32.4" customHeight="1">
       <c r="A21" s="2">
         <v>80</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="21" customHeight="1">
       <c r="A22" s="2">
         <v>81</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="2"/>
-    </row>
-    <row r="23" spans="1:3" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="25.8" customHeight="1">
       <c r="A23" s="2">
         <v>82</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="21.6" customHeight="1">
       <c r="A24" s="2">
         <v>83</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="22.8" customHeight="1">
       <c r="A25" s="2">
         <v>84</v>
       </c>
@@ -783,68 +814,70 @@
         <v>7</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="22.8" customHeight="1">
       <c r="A26" s="2">
         <v>85</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" s="2">
         <v>86</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="26.4" customHeight="1">
       <c r="A28" s="2">
         <v>87</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="21" customHeight="1">
       <c r="A29" s="2">
         <v>88</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" s="2"/>
-    </row>
-    <row r="30" spans="1:3" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="21.6" customHeight="1">
       <c r="A30" s="2">
         <v>89</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="20.399999999999999" customHeight="1">
       <c r="A31" s="2">
         <v>90</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>35</v>

</xml_diff>